<commit_message>
fix circular references in Offer Overview formulas, add PLN formatting, spacer rows, total row
</commit_message>
<xml_diff>
--- a/Kosztorys.xlsx
+++ b/Kosztorys.xlsx
@@ -20,10 +20,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="_([$PLN]\ * #,##0.00_);_([$PLN]\ * \(#,##0.00\);_([$PLN]\ * &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="165" formatCode="#,##0 &quot;PLN&quot;"/>
   </numFmts>
-  <fonts count="17">
+  <fonts count="25">
     <font>
       <name val="Arial"/>
       <color rgb="FF000000"/>
@@ -129,8 +130,54 @@
       <name val="Aptos"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="001A1A1A"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F3864"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001A1A1A"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="001A1A1A"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F3864"/>
+      <sz val="12"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -149,8 +196,32 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F3864"/>
+        <bgColor rgb="001F3864"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
+        <bgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002B5B84"/>
+        <bgColor rgb="002B5B84"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D6E4F0"/>
+        <bgColor rgb="00D6E4F0"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -158,12 +229,70 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00B0B0B0"/>
+      </left>
+      <right style="thin">
+        <color rgb="00B0B0B0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00B0B0B0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00B0B0B0"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00B0B0B0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00B0B0B0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00B0B0B0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00B0B0B0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00B0B0B0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00B0B0B0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00B0B0B0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00B0B0B0"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="9" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="63">
+  <cellXfs count="80">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
@@ -288,6 +417,49 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="19" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="19" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="24" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -568,33 +740,51 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F55"/>
+  <dimension ref="A1:F54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="32" customWidth="1" style="51" min="1" max="1"/>
+    <col width="36" customWidth="1" style="51" min="1" max="1"/>
     <col width="55" customWidth="1" style="51" min="2" max="2"/>
-    <col width="12" customWidth="1" style="51" min="3" max="3"/>
-    <col width="12" customWidth="1" style="51" min="4" max="4"/>
-    <col width="18" customWidth="1" style="51" min="5" max="5"/>
-    <col width="12" customWidth="1" style="51" min="6" max="6"/>
+    <col width="16" customWidth="1" style="51" min="3" max="3"/>
+    <col width="16" customWidth="1" style="51" min="4" max="4"/>
+    <col width="20" customWidth="1" style="51" min="5" max="5"/>
+    <col width="16" customWidth="1" style="51" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="56" t="inlineStr">
+    <row r="1" ht="40" customHeight="1" s="51">
+      <c r="A1" s="63" t="inlineStr">
         <is>
           <t>AI SDLC — Oferta wdrożenia</t>
         </is>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="57" t="inlineStr">
+      <c r="B1" s="64" t="n"/>
+      <c r="C1" s="64" t="n"/>
+      <c r="D1" s="64" t="n"/>
+      <c r="E1" s="64" t="n"/>
+      <c r="F1" s="64" t="n"/>
+    </row>
+    <row r="2" ht="30" customHeight="1" s="51">
+      <c r="A2" s="75" t="n"/>
+      <c r="B2" s="75" t="n"/>
+      <c r="C2" s="75" t="n"/>
+      <c r="D2" s="75" t="n"/>
+      <c r="E2" s="75" t="n"/>
+      <c r="F2" s="75" t="n"/>
+    </row>
+    <row r="3" ht="30" customHeight="1" s="51">
+      <c r="A3" s="65" t="inlineStr">
         <is>
           <t>Executive Summary</t>
         </is>
       </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="58" t="inlineStr">
+      <c r="B3" s="66" t="n"/>
+      <c r="C3" s="66" t="n"/>
+      <c r="D3" s="66" t="n"/>
+      <c r="E3" s="66" t="n"/>
+      <c r="F3" s="66" t="n"/>
+    </row>
+    <row r="4" ht="139" customHeight="1" s="51">
+      <c r="A4" s="67" t="inlineStr">
         <is>
           <t>Bottega proponuje kompleksowe wdrożenie inżynierii oprogramowania wspomaganej sztuczną inteligencją (AI SDLC) w dwóch obszarach biznesowych: Bankowość Centralna oraz Capital Markets, wraz z opcjonalną technologiczną restrukturyzacją wybranych modułów.
 Oferta obejmuje budowę baz wiedzy i dokumentacji zoptymalizowanej pod AI, konfigurację narzędzi i instrukcji dla analityków, developerów i reviewerów, wdrożenie automatyzacji CI/CD oraz security gates, a także szkolenia i transfer know-how.
@@ -602,474 +792,582 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
-    <row r="7">
-      <c r="A7" s="57" t="inlineStr">
+    <row r="5" ht="30" customHeight="1" s="51">
+      <c r="A5" s="75" t="n"/>
+      <c r="B5" s="75" t="n"/>
+      <c r="C5" s="75" t="n"/>
+      <c r="D5" s="75" t="n"/>
+      <c r="E5" s="75" t="n"/>
+      <c r="F5" s="75" t="n"/>
+    </row>
+    <row r="6" ht="30" customHeight="1" s="51">
+      <c r="A6" s="65" t="inlineStr">
         <is>
           <t>Podejście i fazy wdrożenia</t>
         </is>
       </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="58" t="inlineStr">
+      <c r="B6" s="66" t="n"/>
+      <c r="C6" s="66" t="n"/>
+      <c r="D6" s="66" t="n"/>
+      <c r="E6" s="66" t="n"/>
+      <c r="F6" s="66" t="n"/>
+    </row>
+    <row r="7" ht="49" customHeight="1" s="51">
+      <c r="A7" s="67" t="inlineStr">
         <is>
           <t>Nasze podejście to stopniowa ewolucja, a nie rewolucja. Integrujemy AI tam, gdzie przynosi wymierny zwrot z inwestycji i odciąża inżynierów od powtarzalnych zadań, unikając pułapek związanych z bezpieczeństwem, halucynacjami modeli i obniżeniem jakości kodu.</t>
         </is>
       </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="59" t="inlineStr">
+      <c r="B7" s="67" t="n"/>
+    </row>
+    <row r="8" ht="49" customHeight="1" s="51">
+      <c r="A8" s="68" t="inlineStr">
         <is>
           <t>Faza 1 — Audit i strategia</t>
         </is>
       </c>
-      <c r="B9" s="58" t="inlineStr">
+      <c r="B8" s="67" t="inlineStr">
         <is>
           <t>Analiza procesu wytwórczego, stosu technologicznego i kultury inżynierskiej. Identyfikacja obszarów o najwyższym potencjale zwrotu. Wynik: roadmapa wdrożenia.</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="59" t="inlineStr">
+    <row r="9" ht="64" customHeight="1" s="51">
+      <c r="A9" s="69" t="inlineStr">
         <is>
           <t>Faza 2 — Proof of Value</t>
         </is>
       </c>
-      <c r="B10" s="58" t="inlineStr">
-        <is>
-          <t>Pilotaż na wybranym zespole lub module. Praca własna Bottega (przygotowanie narzędzi, dokumentacji) + pair programming online (transfer know-how). Wynik: działające rozwiązanie + udowodniona wartość.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="59" t="inlineStr">
+      <c r="B9" s="70" t="inlineStr">
+        <is>
+          <t>Pilotaż na wybranym zespole lub module. Praca własna Bottega (przygotowanie narzędzi, dokumentacji) + pair programming online (transfer know-how). Wynik: działające rozwiązanie + udowodniona wartość przed skalowaniem.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="49" customHeight="1" s="51">
+      <c r="A10" s="68" t="inlineStr">
         <is>
           <t>Faza 3 — Skalowanie kompetencji</t>
         </is>
       </c>
-      <c r="B11" s="58" t="inlineStr">
+      <c r="B10" s="67" t="inlineStr">
         <is>
           <t>Rozszerzenie praktyk na całą organizację. Przekazanie licencji z bezterminowym prawem do użytku. Szkolenia dla analityków, PM i developerów.</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="57" t="inlineStr">
+    <row r="11" ht="30" customHeight="1" s="51">
+      <c r="A11" s="75" t="n"/>
+      <c r="B11" s="75" t="n"/>
+      <c r="C11" s="75" t="n"/>
+      <c r="D11" s="75" t="n"/>
+      <c r="E11" s="75" t="n"/>
+      <c r="F11" s="75" t="n"/>
+    </row>
+    <row r="12" ht="30" customHeight="1" s="51">
+      <c r="A12" s="65" t="inlineStr">
         <is>
           <t>Zakres wdrożenia</t>
         </is>
       </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="59" t="inlineStr">
+      <c r="B12" s="66" t="n"/>
+      <c r="C12" s="66" t="n"/>
+      <c r="D12" s="66" t="n"/>
+      <c r="E12" s="66" t="n"/>
+      <c r="F12" s="66" t="n"/>
+    </row>
+    <row r="13" ht="124" customHeight="1" s="51">
+      <c r="A13" s="68" t="inlineStr">
         <is>
           <t>TOTAL.01 — Bankowość Centralna — AI SDLC</t>
         </is>
       </c>
-      <c r="B14" s="58" t="inlineStr">
+      <c r="B13" s="67" t="inlineStr">
         <is>
           <t>Pełen zestaw praktyk AI SDLC: skonsolidowanie dokumentacji funkcji systemu (IK.1), mapowanie funkcjonalności na kod i architekturę (IK.2), dokumentacja frontendu i backendu dla AI (IK.4, IK.5), instrukcje AI do analizy regulatorów KNF/UE (EK.1), narzędzia dla analityków i developerów (TL.1–TL.5).
 Efekt: wspólny język z AI, szybsza analiza impaktu, eliminacja błędów z nieaktualnej dokumentacji.</t>
         </is>
       </c>
-      <c r="E14" s="60">
+      <c r="E13" s="76">
         <f>'Central Banking'!H282</f>
         <v/>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="59" t="inlineStr">
+    <row r="14" ht="49" customHeight="1" s="51">
+      <c r="A14" s="69" t="inlineStr">
         <is>
           <t>TOTAL.02 — Capital Markets — AI SDLC</t>
         </is>
       </c>
-      <c r="B15" s="58" t="inlineStr">
+      <c r="B14" s="70" t="inlineStr">
         <is>
           <t>Analogiczny zakres jak TOTAL.01, dostosowany do specyfiki Capital Markets (regulator GPW). Większy wymiar pracy własnej Bottega by odciążyć zespół klienta.</t>
         </is>
       </c>
-      <c r="E15" s="60">
+      <c r="E14" s="77">
         <f>'Capital Markets'!H281</f>
         <v/>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="59" t="inlineStr">
+    <row r="15" ht="79" customHeight="1" s="51">
+      <c r="A15" s="68" t="inlineStr">
         <is>
           <t>TOTAL.03 — Capital Markets — Refaktoryzacja</t>
         </is>
       </c>
-      <c r="B16" s="58" t="inlineStr">
+      <c r="B15" s="67" t="inlineStr">
         <is>
           <t>Standaryzacja CI/CD (Jenkinsfile, shared library), migracja Ant→Maven/Gradle, automatyzacja deploy QA, ujednolicenie artefaktów, iOS build/release (Fastlane), security gates (Fortify, Dependency-Track), plan migracji z wyceną etapową.</t>
         </is>
       </c>
-      <c r="E16" s="60">
+      <c r="E15" s="76">
         <f>'Refactor Capital Markets'!H143</f>
         <v/>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="59" t="inlineStr">
+    <row r="16" ht="49" customHeight="1" s="51">
+      <c r="A16" s="69" t="inlineStr">
         <is>
           <t>TOTAL.04 — Pakiet szkoleń</t>
         </is>
       </c>
-      <c r="B17" s="58" t="inlineStr">
+      <c r="B16" s="70" t="inlineStr">
         <is>
           <t>Szkolenie AI SDLC dla analityków i PM (2 dni) oraz dla developerów (3 dni). Bazuje na realnych zadaniach i kodzie projektów.</t>
         </is>
       </c>
-      <c r="E17" s="60">
-        <f>SUM(E31:E34)</f>
+      <c r="E16" s="77">
+        <f>SUM(Podsumowanie!E31:E34)</f>
         <v/>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="59" t="inlineStr">
+    <row r="17" ht="40" customHeight="1" s="51">
+      <c r="A17" s="68" t="inlineStr">
         <is>
           <t>TOTAL.05 — Gwarancja 1 rok / Bufor</t>
         </is>
       </c>
-      <c r="B18" s="58" t="inlineStr">
+      <c r="B17" s="67" t="inlineStr">
         <is>
           <t>Pakiet dodatkowych godzin na bieżące wsparcie, korekty i niespodziewane wyzwania po wdrożeniu.</t>
         </is>
       </c>
-      <c r="E18" s="60">
-        <f>SUM(E39:E42)</f>
+      <c r="E17" s="76">
+        <f>SUM(Podsumowanie!E39:E42)</f>
         <v/>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="59" t="inlineStr">
+    <row r="18" ht="40" customHeight="1" s="51">
+      <c r="A18" s="69" t="inlineStr">
         <is>
           <t>TOTAL.06 — Narzędzia i licencje</t>
         </is>
       </c>
-      <c r="B19" s="58" t="inlineStr">
+      <c r="B18" s="70" t="inlineStr">
         <is>
           <t>Przekazanie licencji na narzędzia AI SDLC z bezterminowymi prawami do wewnętrznego użytku i własnego rozwoju.</t>
         </is>
       </c>
-      <c r="E19" s="60">
+      <c r="E18" s="77">
         <f>Narzędzia!G86</f>
         <v/>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="57" t="inlineStr">
+    <row r="19" ht="35" customHeight="1" s="51">
+      <c r="A19" s="78" t="inlineStr">
+        <is>
+          <t>Łączna wartość</t>
+        </is>
+      </c>
+      <c r="E19" s="79">
+        <f>SUM(Podsumowanie!E11,Podsumowanie!E19,Podsumowanie!E27,Podsumowanie!E35,Podsumowanie!E43,Podsumowanie!E51)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20" ht="30" customHeight="1" s="51">
+      <c r="A20" s="75" t="n"/>
+      <c r="B20" s="75" t="n"/>
+      <c r="C20" s="75" t="n"/>
+      <c r="D20" s="75" t="n"/>
+      <c r="E20" s="75" t="n"/>
+      <c r="F20" s="75" t="n"/>
+    </row>
+    <row r="21" ht="30" customHeight="1" s="51">
+      <c r="A21" s="65" t="inlineStr">
         <is>
           <t>Efekty biznesowe</t>
         </is>
       </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="59" t="inlineStr">
+      <c r="B21" s="66" t="n"/>
+      <c r="C21" s="66" t="n"/>
+      <c r="D21" s="66" t="n"/>
+      <c r="E21" s="66" t="n"/>
+      <c r="F21" s="66" t="n"/>
+    </row>
+    <row r="22" ht="64" customHeight="1" s="51">
+      <c r="A22" s="68" t="inlineStr">
         <is>
           <t>Przyspieszenie Time-to-Market</t>
         </is>
       </c>
-      <c r="B22" s="58" t="inlineStr">
+      <c r="B22" s="67" t="inlineStr">
         <is>
           <t>Automatyzacja powtarzalnych zadań skraca czas dostarczania funkcjonalności. AI przejmuje żmudne czynności, inżynierowie skupiają się na pracy twórczej.
 → TOTAL.01, TOTAL.02, TOTAL.03</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="59" t="inlineStr">
+    <row r="23" ht="64" customHeight="1" s="51">
+      <c r="A23" s="69" t="inlineStr">
         <is>
           <t>Redukcja długu technicznego</t>
         </is>
       </c>
-      <c r="B23" s="58" t="inlineStr">
+      <c r="B23" s="70" t="inlineStr">
         <is>
           <t>Systematyczna poprawa jakości kodu i architektury przez AI Review (bugs, architektura, complexicity, zgodność ze specyfikacją).
 → TOTAL.03, TOTAL.01, TOTAL.02</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="59" t="inlineStr">
+    <row r="24" ht="79" customHeight="1" s="51">
+      <c r="A24" s="68" t="inlineStr">
         <is>
           <t>Retencja wiedzy projektowej</t>
         </is>
       </c>
-      <c r="B24" s="58" t="inlineStr">
+      <c r="B24" s="67" t="inlineStr">
         <is>
           <t>AI jako "kustosz wiedzy" — skonsolidowana dokumentacja, baza wiedzy mapująca funkcjonalność na kod. Szybsze wdrażanie nowych pracowników, minimalizacja ryzyka utraty wiedzy przy rotacji.
 → TOTAL.01, TOTAL.02, TOTAL.06</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="59" t="inlineStr">
+    <row r="25" ht="64" customHeight="1" s="51">
+      <c r="A25" s="69" t="inlineStr">
         <is>
           <t>Skalowanie kompetencji</t>
         </is>
       </c>
-      <c r="B25" s="58" t="inlineStr">
+      <c r="B25" s="70" t="inlineStr">
         <is>
           <t>Ujednolicenie standardów pracy. Dzięki narzędziom i instrukcjom AI każdy inżynier pracuje według tych samych wzorców.
 → TOTAL.04, TOTAL.01, TOTAL.02</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="59" t="inlineStr">
+    <row r="26" ht="64" customHeight="1" s="51">
+      <c r="A26" s="68" t="inlineStr">
         <is>
           <t>Bezpieczeństwo danych</t>
         </is>
       </c>
-      <c r="B26" s="58" t="inlineStr">
+      <c r="B26" s="67" t="inlineStr">
         <is>
           <t>Pełna kontrola nad kodem źródłowym i dokumentacją. Gating bezpieczeństwa w pipeline. Opcje: Cloud Native, Private Cloud (VPC) lub On-Premise (Air-Gapped).
 → TOTAL.03, TOTAL.06</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="57" t="inlineStr">
+    <row r="27" ht="30" customHeight="1" s="51">
+      <c r="A27" s="75" t="n"/>
+      <c r="B27" s="75" t="n"/>
+      <c r="C27" s="75" t="n"/>
+      <c r="D27" s="75" t="n"/>
+      <c r="E27" s="75" t="n"/>
+      <c r="F27" s="75" t="n"/>
+    </row>
+    <row r="28" ht="30" customHeight="1" s="51">
+      <c r="A28" s="65" t="inlineStr">
         <is>
           <t>Model dostawy</t>
         </is>
       </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="59" t="inlineStr">
-        <is>
-          <t>Formy współpracy</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="61" t="inlineStr">
+      <c r="B28" s="66" t="n"/>
+      <c r="C28" s="66" t="n"/>
+      <c r="D28" s="66" t="n"/>
+      <c r="E28" s="66" t="n"/>
+      <c r="F28" s="66" t="n"/>
+    </row>
+    <row r="29" ht="25" customHeight="1" s="51">
+      <c r="A29" s="71" t="inlineStr">
+        <is>
+          <t>Forma współpracy</t>
+        </is>
+      </c>
+      <c r="B29" s="71" t="inlineStr">
+        <is>
+          <t>Opis</t>
+        </is>
+      </c>
+      <c r="C29" s="71" t="inlineStr">
+        <is>
+          <t>Kiedy stosujemy</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="34" customHeight="1" s="51">
+      <c r="A30" s="67" t="inlineStr">
         <is>
           <t>Praca własna Bottega</t>
         </is>
       </c>
-      <c r="B30" s="61" t="inlineStr">
-        <is>
-          <t>Eksperci Bottega realizują zadania samodzielnie</t>
-        </is>
-      </c>
-      <c r="D30" s="61" t="inlineStr">
+      <c r="B30" s="67" t="inlineStr">
+        <is>
+          <t>Eksperci Bottega realizują zadania samodzielnie, bez angażowania zespołu klienta</t>
+        </is>
+      </c>
+      <c r="C30" s="67" t="inlineStr">
         <is>
           <t>Budowa narzędzi, dokumentacji, instrukcji</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="61" t="inlineStr">
+    <row r="31" ht="34" customHeight="1" s="51">
+      <c r="A31" s="70" t="inlineStr">
         <is>
           <t>Pair programming online</t>
         </is>
       </c>
-      <c r="B31" s="61" t="inlineStr">
-        <is>
-          <t>Wspólna praca eksperta Bottega z inżynierem klienta</t>
-        </is>
-      </c>
-      <c r="D31" s="61" t="inlineStr">
+      <c r="B31" s="70" t="inlineStr">
+        <is>
+          <t>Wspólna praca eksperta Bottega z inżynierem klienta w parach, przekazująca know-how w czasie rzeczywistym</t>
+        </is>
+      </c>
+      <c r="C31" s="70" t="inlineStr">
         <is>
           <t>Transfer kompetencji: context engineering, refactoring, pipeline</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="61" t="inlineStr">
+    <row r="32" ht="34" customHeight="1" s="51">
+      <c r="A32" s="67" t="inlineStr">
         <is>
           <t>Review po stronie klienta</t>
         </is>
       </c>
-      <c r="B32" s="61" t="inlineStr">
-        <is>
-          <t>Klient weryfikuje efekty przed zamknięciem</t>
-        </is>
-      </c>
-      <c r="D32" s="61" t="inlineStr">
-        <is>
-          <t>Każda dostarczona pozycja</t>
+      <c r="B32" s="67" t="inlineStr">
+        <is>
+          <t>Klient weryfikuje efekty prac Bottega, otrzymuje feedback i możliwość korekty</t>
+        </is>
+      </c>
+      <c r="C32" s="67" t="inlineStr">
+        <is>
+          <t>Każda dostarczona pozycja przed zamknięciem</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="68" t="inlineStr">
+        <is>
+          <t>Środowiska docelowe</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="59" t="inlineStr">
-        <is>
-          <t>Środowiska docelowe</t>
+      <c r="B34" s="67" t="inlineStr">
+        <is>
+          <t>Cloud Native (Enterprise API) — dla firm akceptujących przetwarzanie w chmurze z umowami BAA, stawiających na najwyższą inteligencję modeli</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="60" t="inlineStr">
-        <is>
-          <t>Cloud Native (Enterprise API) — dla firm akceptujących chmurę z BAA</t>
+      <c r="B35" s="70" t="inlineStr">
+        <is>
+          <t>Private Cloud (VPC) — dla organizacji wymagających zgodności z regulacjami korporacyjnymi, posiadających infrastrukturę w chmurze publicznej</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="60" t="inlineStr">
-        <is>
-          <t>Private Cloud (VPC) — dla organizacji z regulacjami korporacyjnymi</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="60" t="inlineStr">
-        <is>
-          <t>On-Premise (Air-Gapped) — dla banków i sektora publicznego</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="57" t="inlineStr">
+      <c r="B36" s="67" t="inlineStr">
+        <is>
+          <t>On-Premise (Air-Gapped) — dla banków i sektora publicznego o najwyższym rygorze tajności; obejmuje dobór hardware'u, konfigurację i support</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="30" customHeight="1" s="51">
+      <c r="A37" s="75" t="n"/>
+      <c r="B37" s="75" t="n"/>
+      <c r="C37" s="75" t="n"/>
+      <c r="D37" s="75" t="n"/>
+      <c r="E37" s="75" t="n"/>
+      <c r="F37" s="75" t="n"/>
+    </row>
+    <row r="38" ht="30" customHeight="1" s="51">
+      <c r="A38" s="65" t="inlineStr">
         <is>
           <t>Ryzyka i mitigacje</t>
         </is>
       </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="59" t="inlineStr">
-        <is>
-          <t>Halucynacje modeli AI</t>
-        </is>
-      </c>
-      <c r="B40" s="58" t="inlineStr">
-        <is>
-          <t>Context engineering — budowa precyzyjnego kontekstu dla LLM; instrukcje AI wymuszające weryfikację faktów; human-in-the-loop</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="59" t="inlineStr">
-        <is>
-          <t>Obniżenie jakości kodu</t>
-        </is>
-      </c>
-      <c r="B41" s="58" t="inlineStr">
-        <is>
-          <t>AI Review w pipeline (bugs, architektura, complexicity, zgodność ze specyfikacją); gating security; code review</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="59" t="inlineStr">
-        <is>
-          <t>Wyciek danych / kodu źródłowego</t>
-        </is>
-      </c>
-      <c r="B42" s="58" t="inlineStr">
-        <is>
-          <t>Opcje On-Premise (Air-Gapped) lub Private Cloud (VPC); polityka danych i instrukcje AI wymuszające lokalne przetwarzanie</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="59" t="inlineStr">
-        <is>
-          <t>Odrzucenie przez zespół</t>
-        </is>
-      </c>
-      <c r="B43" s="58" t="inlineStr">
-        <is>
-          <t>Stopniowe wprowadzanie (ewolucja, nie rewolucja); wartość na pilocie; szkolenia i mentoring; odciążenie od powtarzalnych zadań</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="59" t="inlineStr">
-        <is>
-          <t>Ponoszenie zbędnych kosztów</t>
-        </is>
-      </c>
-      <c r="B44" s="58" t="inlineStr">
-        <is>
-          <t>Harness engineering — wyższa jakość przy mniejszych modelach; wycinanie zbędnego outputu i logów; szkolenia z efektywnego korzystania z AI (TOTAL.04)</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="59" t="inlineStr">
-        <is>
-          <t>Uzależnienie od dostawcy</t>
-        </is>
-      </c>
-      <c r="B45" s="58" t="inlineStr">
-        <is>
-          <t>Przekazanie narzędzi i licencji na własność; bezterminowe prawa; transfer know-how przez pair programming</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="57" t="inlineStr">
+      <c r="B38" s="66" t="n"/>
+      <c r="C38" s="66" t="n"/>
+      <c r="D38" s="66" t="n"/>
+      <c r="E38" s="66" t="n"/>
+      <c r="F38" s="66" t="n"/>
+    </row>
+    <row r="39" ht="28" customHeight="1" s="51">
+      <c r="A39" s="72" t="inlineStr">
+        <is>
+          <t>Ryzyko</t>
+        </is>
+      </c>
+      <c r="B39" s="72" t="inlineStr">
+        <is>
+          <t>Mitigacja</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="49" customHeight="1" s="51">
+      <c r="A40" s="67" t="inlineStr">
+        <is>
+          <t>Halucynacje modeli AI — AI generuje nieprawdziwe lub niepoprawne informacje</t>
+        </is>
+      </c>
+      <c r="B40" s="67" t="inlineStr">
+        <is>
+          <t>Context engineering — budowa precyzyjnego kontekstu dla LLM; instrukcje AI wymuszające weryfikację faktów; rola człowieka w pętli (human-in-the-loop)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="64" customHeight="1" s="51">
+      <c r="A41" s="70" t="inlineStr">
+        <is>
+          <t>Obniżenie jakości kodu — AI generuje kod niezgodny ze standardami</t>
+        </is>
+      </c>
+      <c r="B41" s="70" t="inlineStr">
+        <is>
+          <t>AI Review w pipeline (bugs, architektura, complexicity, zgodność ze specyfikacją); gating security (Fortify, Dependency-Track); code review przez doświadczonych inżynierów</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="49" customHeight="1" s="51">
+      <c r="A42" s="67" t="inlineStr">
+        <is>
+          <t>Wyciek danych / kodu źródłowego — wrażliwy kod trafia do publicznych modeli AI</t>
+        </is>
+      </c>
+      <c r="B42" s="67" t="inlineStr">
+        <is>
+          <t>Możliwość deploymentu On-Premise (Air-Gapped); Private Cloud (VPC); polityka danych i instrukcje AI wymuszające lokalne przetwarzanie</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="49" customHeight="1" s="51">
+      <c r="A43" s="70" t="inlineStr">
+        <is>
+          <t>Odrzucenie przez zespół — inżynierowie nie chcą pracować z AI</t>
+        </is>
+      </c>
+      <c r="B43" s="70" t="inlineStr">
+        <is>
+          <t>Stopniowe wprowadzanie (ewolucja, nie rewolucja); pokazanie wartości na pilocie; szkolenia i mentoring; odciążenie od powtarzalnych zadań</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="64" customHeight="1" s="51">
+      <c r="A44" s="67" t="inlineStr">
+        <is>
+          <t>Ponoszenie zbędnych kosztów — niewłaściwe użycie AI przez nieprzeszkolony personel</t>
+        </is>
+      </c>
+      <c r="B44" s="67" t="inlineStr">
+        <is>
+          <t>Harness engineering — znacząco podnosi jakość przy wykorzystaniu mniejszych modeli; oszczędności dzięki wycinaniu zbędnego outputu i logów; szkolenia z efektywnego korzystania z AI (TOTAL.04)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="64" customHeight="1" s="51">
+      <c r="A45" s="70" t="inlineStr">
+        <is>
+          <t>Uzależnienie od dostawcy (vendor lock-in)</t>
+        </is>
+      </c>
+      <c r="B45" s="70" t="inlineStr">
+        <is>
+          <t>Przekazanie narzędzi i licencji na własność; bezterminowe prawa do wewnętrznego użytku i rozwoju; transfer know-how przez pair programming; dokumentacja i instrukcje pozostają w organizacji</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="30" customHeight="1" s="51">
+      <c r="A46" s="75" t="n"/>
+      <c r="B46" s="75" t="n"/>
+      <c r="C46" s="75" t="n"/>
+      <c r="D46" s="75" t="n"/>
+      <c r="E46" s="75" t="n"/>
+      <c r="F46" s="75" t="n"/>
+    </row>
+    <row r="47" ht="30" customHeight="1" s="51">
+      <c r="A47" s="65" t="inlineStr">
         <is>
           <t>Dlaczego Bottega</t>
         </is>
       </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="60" t="inlineStr">
-        <is>
-          <t>Doświadczenie w bankowości konsumenckiej i inwestycyjnej — projekty transformacyjne w sektorze finansowym; znajomość regulacji KNF, GPW i UE</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="60" t="inlineStr">
-        <is>
-          <t>15 lat doświadczenia w szkoleniach i doradztwie dla zespołów deweloperskich</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="60" t="inlineStr">
-        <is>
-          <t>78 aktywnych trenerów o modelu kompetencji Π (Pi) — silny filar techniczny oraz umiejętności miękkie, talent edukacyjny, myślenie strategiczne</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="60" t="inlineStr">
-        <is>
-          <t>Ponad 12 000 przeszkolonych uczestników, 150 dni szkoleń rocznie</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="60" t="inlineStr">
-        <is>
-          <t>43 klientów z branż: finansowa, medyczna, ubezpieczeniowa, energetyczna, zbrojeniowa, e-commerce</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="60" t="inlineStr">
-        <is>
-          <t>Eksperci: Sławomir Sobótka, Jakub Nabrdalik, Łukasz Szydło, Mariusz Gil</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="62" t="inlineStr">
+      <c r="B47" s="66" t="n"/>
+      <c r="C47" s="66" t="n"/>
+      <c r="D47" s="66" t="n"/>
+      <c r="E47" s="66" t="n"/>
+      <c r="F47" s="66" t="n"/>
+    </row>
+    <row r="48" ht="64" customHeight="1" s="51">
+      <c r="A48" s="67" t="inlineStr">
+        <is>
+          <t>• Doświadczenie w bankowości konsumenckiej i inwestycyjnej — projekty transformacyjne w sektorze finansowym; znajomość regulacji KNF, GPW i UE</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="34" customHeight="1" s="51">
+      <c r="A49" s="70" t="inlineStr">
+        <is>
+          <t>• 15 lat doświadczenia w szkoleniach i doradztwie dla zespołów deweloperskich</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="64" customHeight="1" s="51">
+      <c r="A50" s="67" t="inlineStr">
+        <is>
+          <t>• 78 aktywnych trenerów o modelu kompetencji Π (Pi) — silny filar techniczny oraz umiejętności miękkie, talent edukacyjny, myślenie strategiczne</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="34" customHeight="1" s="51">
+      <c r="A51" s="70" t="inlineStr">
+        <is>
+          <t>• Ponad 12 000 przeszkolonych uczestników, 150 dni szkoleń rocznie</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="49" customHeight="1" s="51">
+      <c r="A52" s="67" t="inlineStr">
+        <is>
+          <t>• 43 klientów z branż: finansowa, medyczna, ubezpieczeniowa, energetyczna, zbrojeniowa, e-commerce</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="34" customHeight="1" s="51">
+      <c r="A53" s="70" t="inlineStr">
+        <is>
+          <t>• Eksperci: Sławomir Sobótka, Jakub Nabrdalik, Łukasz Szydło, Mariusz Gil</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="34" customHeight="1" s="51">
+      <c r="A54" s="67" t="inlineStr">
         <is>
           <t>Wybrani klienci: Intel Polska • Orange Polska • Roche Polska • Asseco Polska • Tomtom Polska • Capgemini • Comarch • Luxoft • Motorola • PZU • Tieto • Atos</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="11">
-    <mergeCell ref="A39:F39"/>
+  <mergeCells count="8">
+    <mergeCell ref="A38:F38"/>
     <mergeCell ref="A47:F47"/>
     <mergeCell ref="A28:F28"/>
-    <mergeCell ref="A13:F13"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A8:F8"/>
-    <mergeCell ref="A55:D55"/>
+    <mergeCell ref="A6:F6"/>
+    <mergeCell ref="A12:F12"/>
     <mergeCell ref="A3:F3"/>
-    <mergeCell ref="A4:F5"/>
     <mergeCell ref="A21:F21"/>
-    <mergeCell ref="A7:F7"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1149,13 +1447,13 @@
           <t>Typ do podsumowania</t>
         </is>
       </c>
-      <c r="G4" s="59" t="inlineStr">
+      <c r="G4" s="73" t="inlineStr">
         <is>
           <t>Opis oferty</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1" s="51">
+    <row r="5" ht="109" customHeight="1" s="51">
       <c r="A5" s="15" t="inlineStr">
         <is>
           <t>TOTAL.01</t>
@@ -1173,10 +1471,10 @@
       </c>
       <c r="D5" s="15" t="n"/>
       <c r="F5" s="2" t="n"/>
-      <c r="G5" s="62" t="inlineStr">
+      <c r="G5" s="74" t="inlineStr">
         <is>
           <t>TOTAL.01 — Bankowość Centralna: AI SDLC + Know-How
-Pełen zestaw praktyk AI SDLC: skonsolidowanie dokumentacji funkcji systemu (IK.1), mapowanie funkcjonalności na kod i architekturę (IK.2), dokumentacja frontendu i backendu zoptymalizowana pod AI (IK.4, IK.5), instrukcje AI do analizy regulatorów KNF/UE (EK.1) oraz narzędzia i instrukcje dla analityków i developerów (TL.1–TL.5). Efekt: analitycy i developerzy zyskują wspólny język z AI.</t>
+Pełen zestaw praktyk AI SDLC: skonsolidowanie dokumentacji funkcji systemu (IK.1), mapowanie funkcjonalności na kod i architekturę (IK.2), dokumentacja frontendu i backendu zoptymalizowana pod AI (IK.4, IK.5), instrukcje AI do analizy regulatorów KNF/UE (EK.1) oraz narzędzia i instrukcje dla analityków i developerów (TL.1–TL.5).</t>
         </is>
       </c>
     </row>
@@ -1256,7 +1554,7 @@
       </c>
       <c r="F11" s="2" t="n"/>
     </row>
-    <row r="13" ht="15" customHeight="1" s="51">
+    <row r="13" ht="79" customHeight="1" s="51">
       <c r="A13" s="15" t="inlineStr">
         <is>
           <t>TOTAL.02</t>
@@ -1274,7 +1572,7 @@
       </c>
       <c r="D13" s="15" t="n"/>
       <c r="F13" s="2" t="n"/>
-      <c r="G13" s="62" t="inlineStr">
+      <c r="G13" s="74" t="inlineStr">
         <is>
           <t>TOTAL.02 — Capital Markets: AI SDLC + Know-How
 Analogiczny zakres jak dla Bankowości Centralnej, dostosowany do specyfiki BU Capital Markets (w tym regulator GPW). Większy wymiar pracy własnej Bottega by odciążyć zespół klienta.</t>
@@ -1359,7 +1657,7 @@
       </c>
       <c r="F19" s="2" t="n"/>
     </row>
-    <row r="21" ht="15" customHeight="1" s="51">
+    <row r="21" ht="124" customHeight="1" s="51">
       <c r="A21" s="15" t="inlineStr">
         <is>
           <t>TOTAL.03</t>
@@ -1377,7 +1675,7 @@
       </c>
       <c r="D21" s="15" t="n"/>
       <c r="F21" s="2" t="n"/>
-      <c r="G21" s="62" t="inlineStr">
+      <c r="G21" s="74" t="inlineStr">
         <is>
           <t>TOTAL.03 — Capital Markets: Technologiczna restrukturyzacja
 Standaryzacja CI/CD na Jenkinsfile (REF.1), migracja builda Ant→Maven/Gradle (REF.2), automatyzacja deploy QA (REF.3), ujednolicenie artefaktów (REF.4), iOS build/release przez Fastlane (REF.5), Fortify/Dependency-Track z gatingiem (REF.6), plan migracji z wyceną etapową (REF.RE.1).</t>
@@ -1475,7 +1773,7 @@
       </c>
       <c r="F27" s="2" t="n"/>
     </row>
-    <row r="29" ht="15" customHeight="1" s="51">
+    <row r="29" ht="64" customHeight="1" s="51">
       <c r="A29" s="15" t="inlineStr">
         <is>
           <t>TOTAL.04</t>
@@ -1489,7 +1787,7 @@
       </c>
       <c r="D29" s="15" t="n"/>
       <c r="F29" s="2" t="n"/>
-      <c r="G29" s="62" t="inlineStr">
+      <c r="G29" s="74" t="inlineStr">
         <is>
           <t>TOTAL.04 — Pakiet szkoleń
 Szkolenia dla szerszego grona pracowników: AI SDLC dla analityków i PM (2 dni) oraz dla developerów (3 dni). Bazują na realnych zadaniach i kodzie projektów.</t>
@@ -1572,7 +1870,7 @@
       </c>
       <c r="F35" s="2" t="n"/>
     </row>
-    <row r="37" ht="15" customHeight="1" s="51">
+    <row r="37" ht="49" customHeight="1" s="51">
       <c r="A37" s="15" t="inlineStr">
         <is>
           <t>TOTAL.05</t>
@@ -1586,7 +1884,7 @@
       </c>
       <c r="D37" s="15" t="n"/>
       <c r="F37" s="2" t="n"/>
-      <c r="G37" s="62" t="inlineStr">
+      <c r="G37" s="74" t="inlineStr">
         <is>
           <t>TOTAL.05 — Gwarancja 1 rok / Bufor
 Pakiet dodatkowych godzin na bieżące wsparcie, korekty i niespodziewane wyzwania po wdrożeniu.</t>
@@ -1664,7 +1962,7 @@
       <c r="E44" s="34" t="n"/>
       <c r="F44" s="2" t="n"/>
     </row>
-    <row r="45" ht="15" customHeight="1" s="51">
+    <row r="45" ht="49" customHeight="1" s="51">
       <c r="A45" s="35" t="inlineStr">
         <is>
           <t>TOTAL.06</t>
@@ -1676,7 +1974,7 @@
           <t>Przekazanie narzędzi AI SDLC i licencji</t>
         </is>
       </c>
-      <c r="G45" s="62" t="inlineStr">
+      <c r="G45" s="74" t="inlineStr">
         <is>
           <t>TOTAL.06 — Przekazanie narzędzi i licencji
 Licencje na narzędzia AI SDLC z bezterminowymi prawami do wewnętrznego użytku i własnego rozwoju.</t>
@@ -1853,7 +2151,7 @@
           <t>Suma</t>
         </is>
       </c>
-      <c r="I4" s="59" t="inlineStr">
+      <c r="I4" s="73" t="inlineStr">
         <is>
           <t>Value proposition</t>
         </is>
@@ -1878,7 +2176,7 @@
       <c r="F6" s="3" t="n"/>
       <c r="G6" s="16" t="n"/>
     </row>
-    <row r="7" ht="16" customHeight="1" s="51">
+    <row r="7" ht="64" customHeight="1" s="51">
       <c r="A7" s="7" t="inlineStr">
         <is>
           <t>IK.1</t>
@@ -1902,7 +2200,7 @@
       <c r="E7" s="3" t="n"/>
       <c r="F7" s="3" t="n"/>
       <c r="G7" s="16" t="n"/>
-      <c r="I7" s="62" t="inlineStr">
+      <c r="I7" s="74" t="inlineStr">
         <is>
           <t>Analityk: pewność że AI rozumie aktualny stan systemu. Developer: AI i agenci wiedzą co jest już zaimplementowane. Reviewer: kontekst do oceny impaktu. QA: pełny kontekst systemu.</t>
         </is>
@@ -2009,7 +2307,7 @@
       <c r="G13" s="16" t="n"/>
       <c r="H13" s="28" t="n"/>
     </row>
-    <row r="14" ht="32" customHeight="1" s="51">
+    <row r="14" ht="49" customHeight="1" s="51">
       <c r="A14" s="7" t="inlineStr">
         <is>
           <t>IK.2</t>
@@ -2034,7 +2332,7 @@
       <c r="F14" s="3" t="n"/>
       <c r="G14" s="16" t="n"/>
       <c r="H14" s="28" t="n"/>
-      <c r="I14" s="62" t="inlineStr">
+      <c r="I14" s="74" t="inlineStr">
         <is>
           <t>Analityk: AI wskazuje miejsca zmian po opisie. Developer: wie dokładnie gdzie zmieniać kod. Reviewer: ocenia pełen impact. QA: wie co testować.</t>
         </is>
@@ -2141,7 +2439,7 @@
       <c r="G20" s="16" t="n"/>
       <c r="H20" s="28" t="n"/>
     </row>
-    <row r="21" ht="32" customHeight="1" s="51">
+    <row r="21" ht="34" customHeight="1" s="51">
       <c r="A21" s="7" t="inlineStr">
         <is>
           <t>IK.3</t>
@@ -2166,7 +2464,7 @@
       <c r="F21" s="3" t="n"/>
       <c r="G21" s="16" t="n"/>
       <c r="H21" s="28" t="n"/>
-      <c r="I21" s="62" t="inlineStr">
+      <c r="I21" s="74" t="inlineStr">
         <is>
           <t>Liderzy: estymaty oparte na wartościach eksperckich.</t>
         </is>
@@ -2273,7 +2571,7 @@
       <c r="G27" s="16" t="n"/>
       <c r="H27" s="28" t="n"/>
     </row>
-    <row r="28" ht="16" customHeight="1" s="51">
+    <row r="28" ht="49" customHeight="1" s="51">
       <c r="A28" s="7" t="inlineStr">
         <is>
           <t>IK.4</t>
@@ -2298,7 +2596,7 @@
       <c r="F28" s="3" t="n"/>
       <c r="G28" s="16" t="n"/>
       <c r="H28" s="28" t="n"/>
-      <c r="I28" s="62" t="inlineStr">
+      <c r="I28" s="74" t="inlineStr">
         <is>
           <t>Analityk: szybsza ocena impaktu na frontend. Developer: AI generuje kod zgodny z architekturą. Reviewer: zgodność z zasadami. QA: spójne testy UI.</t>
         </is>
@@ -2405,7 +2703,7 @@
       <c r="G34" s="16" t="n"/>
       <c r="H34" s="28" t="n"/>
     </row>
-    <row r="35" ht="16" customHeight="1" s="51">
+    <row r="35" ht="64" customHeight="1" s="51">
       <c r="A35" s="7" t="inlineStr">
         <is>
           <t>IK.5</t>
@@ -2430,7 +2728,7 @@
       <c r="F35" s="3" t="n"/>
       <c r="G35" s="16" t="n"/>
       <c r="H35" s="28" t="n"/>
-      <c r="I35" s="62" t="inlineStr">
+      <c r="I35" s="74" t="inlineStr">
         <is>
           <t>Analityk: szybsza ocena impaktu na backend. Developer: AI generuje kod zgodny z wzorcami backendu. Reviewer: zgodność architektoniczna. QA: testy zgodne ze wzorcami.</t>
         </is>
@@ -2537,7 +2835,7 @@
       <c r="G41" s="16" t="n"/>
       <c r="H41" s="28" t="n"/>
     </row>
-    <row r="42" ht="32" customHeight="1" s="51">
+    <row r="42" ht="49" customHeight="1" s="51">
       <c r="A42" s="36" t="inlineStr">
         <is>
           <t>IK.7</t>
@@ -2562,7 +2860,7 @@
       <c r="F42" s="38" t="n"/>
       <c r="G42" s="39" t="n"/>
       <c r="H42" s="40" t="n"/>
-      <c r="I42" s="62" t="inlineStr">
+      <c r="I42" s="74" t="inlineStr">
         <is>
           <t>Analityk: brakujące scenariusze z AI. Developer: scenariusze z danymi. Reviewer: sprawdza pokrycie. QA: gotowe e2e.</t>
         </is>
@@ -2673,7 +2971,7 @@
       <c r="G48" s="16" t="n"/>
       <c r="H48" s="28" t="n"/>
     </row>
-    <row r="49" ht="16" customHeight="1" s="51">
+    <row r="49" ht="49" customHeight="1" s="51">
       <c r="A49" s="7" t="inlineStr">
         <is>
           <t>EK.1</t>
@@ -2698,7 +2996,7 @@
       <c r="F49" s="3" t="n"/>
       <c r="G49" s="16" t="n"/>
       <c r="H49" s="28" t="n"/>
-      <c r="I49" s="62" t="inlineStr">
+      <c r="I49" s="74" t="inlineStr">
         <is>
           <t>Analityk: AI rozbudowuje wymagania regulacyjne, generuje pytania doprecyzowujące, weryfikuje analizę vs źródła.</t>
         </is>
@@ -2805,7 +3103,7 @@
       <c r="G55" s="16" t="n"/>
       <c r="H55" s="28" t="n"/>
     </row>
-    <row r="56" ht="32" customHeight="1" s="51">
+    <row r="56" ht="34" customHeight="1" s="51">
       <c r="A56" s="7" t="inlineStr">
         <is>
           <t>TL.1</t>
@@ -2830,7 +3128,7 @@
       <c r="F56" s="3" t="n"/>
       <c r="G56" s="16" t="n"/>
       <c r="H56" s="28" t="n"/>
-      <c r="I56" s="62" t="inlineStr">
+      <c r="I56" s="74" t="inlineStr">
         <is>
           <t>Analityk: dedykowane środowisko AI do analizy i review dokumentów.</t>
         </is>
@@ -9115,7 +9413,7 @@
           <t>Suma</t>
         </is>
       </c>
-      <c r="I4" s="59" t="inlineStr">
+      <c r="I4" s="73" t="inlineStr">
         <is>
           <t>Value proposition</t>
         </is>
@@ -9129,7 +9427,7 @@
       <c r="E5" s="30" t="n"/>
       <c r="F5" s="3" t="n"/>
     </row>
-    <row r="6" ht="16" customHeight="1" s="51">
+    <row r="6" ht="64" customHeight="1" s="51">
       <c r="A6" s="7" t="inlineStr">
         <is>
           <t>IK.1</t>
@@ -9152,7 +9450,7 @@
       </c>
       <c r="E6" s="30" t="n"/>
       <c r="F6" s="3" t="n"/>
-      <c r="I6" s="62" t="inlineStr">
+      <c r="I6" s="74" t="inlineStr">
         <is>
           <t>Analityk: pewność że AI rozumie aktualny stan systemu. Developer: AI i agenci wiedzą co jest już zaimplementowane. Reviewer: kontekst do oceny impaktu. QA: pełny kontekst systemu.</t>
         </is>
@@ -9251,7 +9549,7 @@
       <c r="E12" s="30" t="n"/>
       <c r="F12" s="3" t="n"/>
     </row>
-    <row r="13" ht="32" customHeight="1" s="51">
+    <row r="13" ht="49" customHeight="1" s="51">
       <c r="A13" s="7" t="inlineStr">
         <is>
           <t>IK.2</t>
@@ -9274,7 +9572,7 @@
       </c>
       <c r="E13" s="30" t="n"/>
       <c r="F13" s="3" t="n"/>
-      <c r="I13" s="62" t="inlineStr">
+      <c r="I13" s="74" t="inlineStr">
         <is>
           <t>Analityk: AI wskazuje miejsca zmian po opisie. Developer: wie dokładnie gdzie zmieniać kod. Reviewer: ocenia pełen impact. QA: wie co testować.</t>
         </is>
@@ -9373,7 +9671,7 @@
       <c r="E19" s="30" t="n"/>
       <c r="F19" s="3" t="n"/>
     </row>
-    <row r="20" ht="32" customHeight="1" s="51">
+    <row r="20" ht="34" customHeight="1" s="51">
       <c r="A20" s="7" t="inlineStr">
         <is>
           <t>IK.3</t>
@@ -9396,7 +9694,7 @@
       </c>
       <c r="E20" s="30" t="n"/>
       <c r="F20" s="3" t="n"/>
-      <c r="I20" s="62" t="inlineStr">
+      <c r="I20" s="74" t="inlineStr">
         <is>
           <t>Liderzy: estymaty oparte na wartościach eksperckich.</t>
         </is>
@@ -9495,7 +9793,7 @@
       <c r="E26" s="30" t="n"/>
       <c r="F26" s="3" t="n"/>
     </row>
-    <row r="27" ht="16" customHeight="1" s="51">
+    <row r="27" ht="49" customHeight="1" s="51">
       <c r="A27" s="7" t="inlineStr">
         <is>
           <t>IK.4</t>
@@ -9518,7 +9816,7 @@
       </c>
       <c r="E27" s="30" t="n"/>
       <c r="F27" s="3" t="n"/>
-      <c r="I27" s="62" t="inlineStr">
+      <c r="I27" s="74" t="inlineStr">
         <is>
           <t>Analityk: szybsza ocena impaktu na frontend. Developer: AI generuje kod zgodny z architekturą. Reviewer: zgodność z zasadami. QA: spójne testy UI.</t>
         </is>
@@ -9617,7 +9915,7 @@
       <c r="E33" s="30" t="n"/>
       <c r="F33" s="3" t="n"/>
     </row>
-    <row r="34" ht="16" customHeight="1" s="51">
+    <row r="34" ht="64" customHeight="1" s="51">
       <c r="A34" s="7" t="inlineStr">
         <is>
           <t>IK.5</t>
@@ -9640,7 +9938,7 @@
       </c>
       <c r="E34" s="30" t="n"/>
       <c r="F34" s="3" t="n"/>
-      <c r="I34" s="62" t="inlineStr">
+      <c r="I34" s="74" t="inlineStr">
         <is>
           <t>Analityk: szybsza ocena impaktu na backend. Developer: AI generuje kod zgodny z wzorcami backendu. Reviewer: zgodność architektoniczna. QA: testy zgodne ze wzorcami.</t>
         </is>
@@ -9739,7 +10037,7 @@
       <c r="E40" s="30" t="n"/>
       <c r="F40" s="3" t="n"/>
     </row>
-    <row r="41" ht="32" customHeight="1" s="51">
+    <row r="41" ht="49" customHeight="1" s="51">
       <c r="A41" s="36" t="inlineStr">
         <is>
           <t>IK.7</t>
@@ -9764,7 +10062,7 @@
       <c r="F41" s="38" t="n"/>
       <c r="G41" s="46" t="n"/>
       <c r="H41" s="46" t="n"/>
-      <c r="I41" s="62" t="inlineStr">
+      <c r="I41" s="74" t="inlineStr">
         <is>
           <t>Analityk: brakujące scenariusze z AI. Developer: scenariusze z danymi. Reviewer: sprawdza pokrycie. QA: gotowe e2e.</t>
         </is>
@@ -9873,7 +10171,7 @@
       <c r="E47" s="30" t="n"/>
       <c r="F47" s="3" t="n"/>
     </row>
-    <row r="48" ht="16" customHeight="1" s="51">
+    <row r="48" ht="34" customHeight="1" s="51">
       <c r="A48" s="7" t="inlineStr">
         <is>
           <t>EK.1</t>
@@ -9896,7 +10194,7 @@
       </c>
       <c r="E48" s="30" t="n"/>
       <c r="F48" s="3" t="n"/>
-      <c r="I48" s="62" t="inlineStr">
+      <c r="I48" s="74" t="inlineStr">
         <is>
           <t>Analityk: AI rozbudowuje wymagania regulacyjne KNF/GPW, generuje pytania, weryfikuje analizę.</t>
         </is>
@@ -9995,7 +10293,7 @@
       <c r="E54" s="30" t="n"/>
       <c r="F54" s="3" t="n"/>
     </row>
-    <row r="55" ht="32" customHeight="1" s="51">
+    <row r="55" ht="34" customHeight="1" s="51">
       <c r="A55" s="7" t="inlineStr">
         <is>
           <t>TL.1</t>
@@ -10018,7 +10316,7 @@
       </c>
       <c r="E55" s="30" t="n"/>
       <c r="F55" s="3" t="n"/>
-      <c r="I55" s="62" t="inlineStr">
+      <c r="I55" s="74" t="inlineStr">
         <is>
           <t>Analityk: dedykowane środowisko AI do analizy i review dokumentów.</t>
         </is>
@@ -13957,13 +14255,13 @@
           <t>Suma</t>
         </is>
       </c>
-      <c r="I4" s="59" t="inlineStr">
+      <c r="I4" s="73" t="inlineStr">
         <is>
           <t>Value proposition</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="15.75" customHeight="1" s="51">
+    <row r="5" ht="34" customHeight="1" s="51">
       <c r="A5" s="15" t="inlineStr">
         <is>
           <t>REF.RE.1</t>
@@ -13986,7 +14284,7 @@
       </c>
       <c r="E5" s="19" t="n"/>
       <c r="F5" s="2" t="n"/>
-      <c r="I5" s="62" t="inlineStr">
+      <c r="I5" s="74" t="inlineStr">
         <is>
           <t>Klient: realny plan migracji z etapami i wyceną zamiast estymacji w ciemno.</t>
         </is>
@@ -14114,7 +14412,7 @@
       <c r="F13" s="2" t="n"/>
       <c r="G13" s="28" t="n"/>
     </row>
-    <row r="14" ht="15.75" customHeight="1" s="51">
+    <row r="14" ht="34" customHeight="1" s="51">
       <c r="A14" s="15" t="inlineStr">
         <is>
           <t>REF.1</t>
@@ -14138,7 +14436,7 @@
       <c r="E14" s="19" t="n"/>
       <c r="F14" s="2" t="n"/>
       <c r="G14" s="28" t="n"/>
-      <c r="I14" s="62" t="inlineStr">
+      <c r="I14" s="74" t="inlineStr">
         <is>
           <t>Developer + AI: jeden znajomy flow CI/CD dla wszystkich repozytoriów.</t>
         </is>
@@ -14258,7 +14556,7 @@
       <c r="F21" s="2" t="n"/>
       <c r="G21" s="28" t="n"/>
     </row>
-    <row r="22" ht="15.75" customHeight="1" s="51">
+    <row r="22" ht="34" customHeight="1" s="51">
       <c r="A22" s="15" t="inlineStr">
         <is>
           <t>REF.2</t>
@@ -14282,7 +14580,7 @@
       <c r="E22" s="19" t="n"/>
       <c r="F22" s="2" t="n"/>
       <c r="G22" s="28" t="n"/>
-      <c r="I22" s="62" t="inlineStr">
+      <c r="I22" s="74" t="inlineStr">
         <is>
           <t>Developer: szybsze buildy, dependency management, security scanning.</t>
         </is>
@@ -14402,7 +14700,7 @@
       <c r="F29" s="2" t="n"/>
       <c r="G29" s="28" t="n"/>
     </row>
-    <row r="30" ht="15.75" customHeight="1" s="51">
+    <row r="30" ht="34" customHeight="1" s="51">
       <c r="A30" s="15" t="inlineStr">
         <is>
           <t>REF.3</t>
@@ -14426,7 +14724,7 @@
       <c r="E30" s="19" t="n"/>
       <c r="F30" s="2" t="n"/>
       <c r="G30" s="28" t="n"/>
-      <c r="I30" s="62" t="inlineStr">
+      <c r="I30" s="74" t="inlineStr">
         <is>
           <t>Developer: self-service deploy, rollback. Koniec wąskiego gardła.</t>
         </is>
@@ -14546,7 +14844,7 @@
       <c r="F37" s="2" t="n"/>
       <c r="G37" s="28" t="n"/>
     </row>
-    <row r="38" ht="15.75" customHeight="1" s="51">
+    <row r="38" ht="34" customHeight="1" s="51">
       <c r="A38" s="15" t="inlineStr">
         <is>
           <t>REF.4</t>
@@ -14570,7 +14868,7 @@
       <c r="E38" s="19" t="n"/>
       <c r="F38" s="2" t="n"/>
       <c r="G38" s="28" t="n"/>
-      <c r="I38" s="62" t="inlineStr">
+      <c r="I38" s="74" t="inlineStr">
         <is>
           <t>Tech lead: w każdej chwili wiadomo co i kiedy trafiło na środowisko.</t>
         </is>
@@ -14688,7 +14986,7 @@
       <c r="F45" s="2" t="n"/>
       <c r="G45" s="28" t="n"/>
     </row>
-    <row r="46" ht="15.75" customHeight="1" s="51">
+    <row r="46" ht="34" customHeight="1" s="51">
       <c r="A46" s="15" t="inlineStr">
         <is>
           <t>REF.5</t>
@@ -14712,7 +15010,7 @@
       <c r="E46" s="19" t="n"/>
       <c r="F46" s="2" t="n"/>
       <c r="G46" s="28" t="n"/>
-      <c r="I46" s="62" t="inlineStr">
+      <c r="I46" s="74" t="inlineStr">
         <is>
           <t>iOS developer: build i podpisywanie w pipeline. Koniec ręcznych obejść.</t>
         </is>
@@ -14832,7 +15130,7 @@
       <c r="F53" s="2" t="n"/>
       <c r="G53" s="28" t="n"/>
     </row>
-    <row r="54" ht="15.75" customHeight="1" s="51">
+    <row r="54" ht="34" customHeight="1" s="51">
       <c r="A54" s="15" t="inlineStr">
         <is>
           <t>REF.6</t>
@@ -14856,7 +15154,7 @@
       <c r="E54" s="19" t="n"/>
       <c r="F54" s="2" t="n"/>
       <c r="G54" s="28" t="n"/>
-      <c r="I54" s="62" t="inlineStr">
+      <c r="I54" s="74" t="inlineStr">
         <is>
           <t>Security: stałe skany SAST/SCA jako warunki blokujące w pipeline.</t>
         </is>
@@ -18610,13 +18908,13 @@
           <t>Suma</t>
         </is>
       </c>
-      <c r="I4" s="59" t="inlineStr">
+      <c r="I4" s="73" t="inlineStr">
         <is>
           <t>Value proposition</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1" s="51">
+    <row r="5" ht="34" customHeight="1" s="51">
       <c r="A5" s="7" t="inlineStr">
         <is>
           <t>RE.1</t>
@@ -18640,7 +18938,7 @@
       <c r="E5" s="3" t="n"/>
       <c r="F5" s="3" t="n"/>
       <c r="G5" s="16" t="n"/>
-      <c r="I5" s="62" t="inlineStr">
+      <c r="I5" s="74" t="inlineStr">
         <is>
           <t>Rekomendacje narzędzi AI dopasowane do istniejących subskrypcji i infrastruktury.</t>
         </is>
@@ -18666,7 +18964,7 @@
       </c>
       <c r="H6" s="28" t="n"/>
     </row>
-    <row r="7" ht="15" customHeight="1" s="51">
+    <row r="7" ht="34" customHeight="1" s="51">
       <c r="A7" s="7" t="inlineStr">
         <is>
           <t>IK.1</t>
@@ -18691,7 +18989,7 @@
       <c r="F7" s="3" t="n"/>
       <c r="G7" s="16" t="n"/>
       <c r="H7" s="28" t="n"/>
-      <c r="I7" s="62" t="inlineStr">
+      <c r="I7" s="74" t="inlineStr">
         <is>
           <t>Narzędzie do konsolidacji dokumentacji funkcji systemu dla AI.</t>
         </is>
@@ -18716,7 +19014,7 @@
       </c>
       <c r="H8" s="28" t="n"/>
     </row>
-    <row r="9" ht="15" customHeight="1" s="51">
+    <row r="9" ht="34" customHeight="1" s="51">
       <c r="A9" s="7" t="inlineStr">
         <is>
           <t>IK.2</t>
@@ -18741,7 +19039,7 @@
       <c r="F9" s="3" t="n"/>
       <c r="G9" s="16" t="n"/>
       <c r="H9" s="28" t="n"/>
-      <c r="I9" s="62" t="inlineStr">
+      <c r="I9" s="74" t="inlineStr">
         <is>
           <t>Narzędzie mapowania funkcjonalności na kod i architekturę.</t>
         </is>
@@ -18766,7 +19064,7 @@
       </c>
       <c r="H10" s="28" t="n"/>
     </row>
-    <row r="11" ht="15" customHeight="1" s="51">
+    <row r="11" ht="34" customHeight="1" s="51">
       <c r="A11" s="7" t="inlineStr">
         <is>
           <t>IK.3</t>
@@ -18791,7 +19089,7 @@
       <c r="F11" s="3" t="n"/>
       <c r="G11" s="16" t="n"/>
       <c r="H11" s="28" t="n"/>
-      <c r="I11" s="62" t="inlineStr">
+      <c r="I11" s="74" t="inlineStr">
         <is>
           <t>Narzędzie heurystycznego szacowania pracochłonności.</t>
         </is>
@@ -18816,7 +19114,7 @@
       </c>
       <c r="H12" s="28" t="n"/>
     </row>
-    <row r="13" ht="15" customHeight="1" s="51">
+    <row r="13" ht="34" customHeight="1" s="51">
       <c r="A13" s="7" t="inlineStr">
         <is>
           <t>IK.4</t>
@@ -18841,7 +19139,7 @@
       <c r="F13" s="3" t="n"/>
       <c r="G13" s="16" t="n"/>
       <c r="H13" s="28" t="n"/>
-      <c r="I13" s="62" t="inlineStr">
+      <c r="I13" s="74" t="inlineStr">
         <is>
           <t>Narzędzie dokumentacji architektury frontendu dla AI.</t>
         </is>
@@ -18866,7 +19164,7 @@
       </c>
       <c r="H14" s="28" t="n"/>
     </row>
-    <row r="15" ht="15" customHeight="1" s="51">
+    <row r="15" ht="34" customHeight="1" s="51">
       <c r="A15" s="7" t="inlineStr">
         <is>
           <t>IK.5</t>
@@ -18891,7 +19189,7 @@
       <c r="F15" s="3" t="n"/>
       <c r="G15" s="16" t="n"/>
       <c r="H15" s="28" t="n"/>
-      <c r="I15" s="62" t="inlineStr">
+      <c r="I15" s="74" t="inlineStr">
         <is>
           <t>Narzędzie dokumentacji architektury backendu dla AI.</t>
         </is>
@@ -18916,7 +19214,7 @@
       </c>
       <c r="H16" s="28" t="n"/>
     </row>
-    <row r="17" ht="15" customHeight="1" s="51">
+    <row r="17" ht="20" customHeight="1" s="51">
       <c r="A17" s="7" t="inlineStr">
         <is>
           <t>IK.7</t>
@@ -18941,7 +19239,7 @@
       <c r="F17" s="3" t="n"/>
       <c r="G17" s="16" t="n"/>
       <c r="H17" s="28" t="n"/>
-      <c r="I17" s="62" t="inlineStr">
+      <c r="I17" s="74" t="inlineStr">
         <is>
           <t>Narzędzie implementacji scenariuszy e2e.</t>
         </is>
@@ -18966,7 +19264,7 @@
       </c>
       <c r="H18" s="28" t="n"/>
     </row>
-    <row r="19" ht="15" customHeight="1" s="51">
+    <row r="19" ht="34" customHeight="1" s="51">
       <c r="A19" s="7" t="inlineStr">
         <is>
           <t>EK.1</t>
@@ -18991,7 +19289,7 @@
       <c r="F19" s="3" t="n"/>
       <c r="G19" s="16" t="n"/>
       <c r="H19" s="28" t="n"/>
-      <c r="I19" s="62" t="inlineStr">
+      <c r="I19" s="74" t="inlineStr">
         <is>
           <t>Narzędzie AI do pracy ze źródłami regulatorów KNF/UE.</t>
         </is>
@@ -19016,7 +19314,7 @@
       </c>
       <c r="H20" s="28" t="n"/>
     </row>
-    <row r="21" ht="15" customHeight="1" s="51">
+    <row r="21" ht="20" customHeight="1" s="51">
       <c r="A21" s="7" t="inlineStr">
         <is>
           <t>TL.1</t>
@@ -19041,7 +19339,7 @@
       <c r="F21" s="3" t="n"/>
       <c r="G21" s="16" t="n"/>
       <c r="H21" s="28" t="n"/>
-      <c r="I21" s="62" t="inlineStr">
+      <c r="I21" s="74" t="inlineStr">
         <is>
           <t>Środowisko AI dla analityków.</t>
         </is>
@@ -19066,7 +19364,7 @@
       </c>
       <c r="H22" s="28" t="n"/>
     </row>
-    <row r="23" ht="15" customHeight="1" s="51">
+    <row r="23" ht="20" customHeight="1" s="51">
       <c r="A23" s="7" t="inlineStr">
         <is>
           <t>TL.2</t>
@@ -19091,7 +19389,7 @@
       <c r="F23" s="3" t="n"/>
       <c r="G23" s="16" t="n"/>
       <c r="H23" s="28" t="n"/>
-      <c r="I23" s="62" t="inlineStr">
+      <c r="I23" s="74" t="inlineStr">
         <is>
           <t>Instrukcje AI do gap analysis i spike analysis.</t>
         </is>
@@ -19116,7 +19414,7 @@
       </c>
       <c r="H24" s="28" t="n"/>
     </row>
-    <row r="25" ht="15" customHeight="1" s="51">
+    <row r="25" ht="20" customHeight="1" s="51">
       <c r="A25" s="7" t="inlineStr">
         <is>
           <t>TL.2.1</t>
@@ -19141,7 +19439,7 @@
       <c r="F25" s="3" t="n"/>
       <c r="G25" s="16" t="n"/>
       <c r="H25" s="28" t="n"/>
-      <c r="I25" s="62" t="inlineStr">
+      <c r="I25" s="74" t="inlineStr">
         <is>
           <t>Instrukcje AI do review analizy vs KNF/UE.</t>
         </is>
@@ -19166,7 +19464,7 @@
       </c>
       <c r="H26" s="28" t="n"/>
     </row>
-    <row r="27" ht="15" customHeight="1" s="51">
+    <row r="27" ht="20" customHeight="1" s="51">
       <c r="A27" s="7" t="inlineStr">
         <is>
           <t>TL.3</t>
@@ -19191,7 +19489,7 @@
       <c r="F27" s="3" t="n"/>
       <c r="G27" s="16" t="n"/>
       <c r="H27" s="28" t="n"/>
-      <c r="I27" s="62" t="inlineStr">
+      <c r="I27" s="74" t="inlineStr">
         <is>
           <t>Generowanie diagramów BPMN/UML z AI.</t>
         </is>
@@ -19216,7 +19514,7 @@
       </c>
       <c r="H28" s="28" t="n"/>
     </row>
-    <row r="29" ht="15" customHeight="1" s="51">
+    <row r="29" ht="20" customHeight="1" s="51">
       <c r="A29" s="7" t="inlineStr">
         <is>
           <t>TL.4</t>
@@ -19241,7 +19539,7 @@
       <c r="F29" s="3" t="n"/>
       <c r="G29" s="16" t="n"/>
       <c r="H29" s="28" t="n"/>
-      <c r="I29" s="62" t="inlineStr">
+      <c r="I29" s="74" t="inlineStr">
         <is>
           <t>Generowanie UI/UX low fidelity z AI.</t>
         </is>
@@ -19266,7 +19564,7 @@
       </c>
       <c r="H30" s="28" t="n"/>
     </row>
-    <row r="31" ht="15" customHeight="1" s="51">
+    <row r="31" ht="20" customHeight="1" s="51">
       <c r="A31" s="7" t="inlineStr">
         <is>
           <t>TL.5</t>
@@ -19291,7 +19589,7 @@
       <c r="F31" s="3" t="n"/>
       <c r="G31" s="16" t="n"/>
       <c r="H31" s="28" t="n"/>
-      <c r="I31" s="62" t="inlineStr">
+      <c r="I31" s="74" t="inlineStr">
         <is>
           <t>AI proponuje scenariusze testowe z analizy.</t>
         </is>
@@ -19316,7 +19614,7 @@
       </c>
       <c r="H32" s="28" t="n"/>
     </row>
-    <row r="33" ht="15" customHeight="1" s="51">
+    <row r="33" ht="20" customHeight="1" s="51">
       <c r="A33" s="7" t="inlineStr">
         <is>
           <t>TL.29</t>
@@ -19341,7 +19639,7 @@
       <c r="F33" s="3" t="n"/>
       <c r="G33" s="16" t="n"/>
       <c r="H33" s="28" t="n"/>
-      <c r="I33" s="62" t="inlineStr">
+      <c r="I33" s="74" t="inlineStr">
         <is>
           <t>Integracja z Enterprise Architect.</t>
         </is>
@@ -19366,7 +19664,7 @@
       </c>
       <c r="H34" s="28" t="n"/>
     </row>
-    <row r="35" ht="15" customHeight="1" s="51">
+    <row r="35" ht="20" customHeight="1" s="51">
       <c r="A35" s="7" t="inlineStr">
         <is>
           <t>TL.30</t>
@@ -19391,7 +19689,7 @@
       <c r="F35" s="3" t="n"/>
       <c r="G35" s="16" t="n"/>
       <c r="H35" s="28" t="n"/>
-      <c r="I35" s="62" t="inlineStr">
+      <c r="I35" s="74" t="inlineStr">
         <is>
           <t>Formatowanie specyfikacji dla AI.</t>
         </is>
@@ -19459,7 +19757,7 @@
       </c>
       <c r="H38" s="28" t="n"/>
     </row>
-    <row r="39" ht="15" customHeight="1" s="51">
+    <row r="39" ht="20" customHeight="1" s="51">
       <c r="A39" s="7" t="inlineStr">
         <is>
           <t>TL.9</t>
@@ -19484,7 +19782,7 @@
       <c r="F39" s="3" t="n"/>
       <c r="G39" s="16" t="n"/>
       <c r="H39" s="28" t="n"/>
-      <c r="I39" s="62" t="inlineStr">
+      <c r="I39" s="74" t="inlineStr">
         <is>
           <t>AI odpyta bazę Oracle (readonly).</t>
         </is>
@@ -19509,7 +19807,7 @@
       </c>
       <c r="H40" s="28" t="n"/>
     </row>
-    <row r="41" ht="15" customHeight="1" s="51">
+    <row r="41" ht="20" customHeight="1" s="51">
       <c r="A41" s="7" t="inlineStr">
         <is>
           <t>TL.10</t>
@@ -19534,7 +19832,7 @@
       <c r="F41" s="3" t="n"/>
       <c r="G41" s="16" t="n"/>
       <c r="H41" s="28" t="n"/>
-      <c r="I41" s="62" t="inlineStr">
+      <c r="I41" s="74" t="inlineStr">
         <is>
           <t>Reverse engineering zasad architektonicznych.</t>
         </is>
@@ -19559,7 +19857,7 @@
       </c>
       <c r="H42" s="28" t="n"/>
     </row>
-    <row r="43" ht="15" customHeight="1" s="51">
+    <row r="43" ht="20" customHeight="1" s="51">
       <c r="A43" s="7" t="inlineStr">
         <is>
           <t>TL.13</t>
@@ -19584,7 +19882,7 @@
       <c r="F43" s="3" t="n"/>
       <c r="G43" s="16" t="n"/>
       <c r="H43" s="28" t="n"/>
-      <c r="I43" s="62" t="inlineStr">
+      <c r="I43" s="74" t="inlineStr">
         <is>
           <t>AI robi hot swap, redeploy, podgląda logi.</t>
         </is>
@@ -19609,7 +19907,7 @@
       </c>
       <c r="H44" s="28" t="n"/>
     </row>
-    <row r="45" ht="15" customHeight="1" s="51">
+    <row r="45" ht="20" customHeight="1" s="51">
       <c r="A45" s="7" t="inlineStr">
         <is>
           <t>TL.14</t>
@@ -19634,7 +19932,7 @@
       <c r="F45" s="3" t="n"/>
       <c r="G45" s="16" t="n"/>
       <c r="H45" s="28" t="n"/>
-      <c r="I45" s="62" t="inlineStr">
+      <c r="I45" s="74" t="inlineStr">
         <is>
           <t>AI uruchamia pipeline Jenkins.</t>
         </is>
@@ -19659,7 +19957,7 @@
       </c>
       <c r="H46" s="28" t="n"/>
     </row>
-    <row r="47" ht="15" customHeight="1" s="51">
+    <row r="47" ht="20" customHeight="1" s="51">
       <c r="A47" s="7" t="inlineStr">
         <is>
           <t>TL.31</t>
@@ -19684,7 +19982,7 @@
       <c r="F47" s="3" t="n"/>
       <c r="G47" s="16" t="n"/>
       <c r="H47" s="28" t="n"/>
-      <c r="I47" s="62" t="inlineStr">
+      <c r="I47" s="74" t="inlineStr">
         <is>
           <t>AI lokalny troubleshooting.</t>
         </is>
@@ -19709,7 +20007,7 @@
       </c>
       <c r="H48" s="28" t="n"/>
     </row>
-    <row r="49" ht="15" customHeight="1" s="51">
+    <row r="49" ht="20" customHeight="1" s="51">
       <c r="A49" s="7" t="inlineStr">
         <is>
           <t>TL.32</t>
@@ -19734,7 +20032,7 @@
       <c r="F49" s="3" t="n"/>
       <c r="G49" s="16" t="n"/>
       <c r="H49" s="28" t="n"/>
-      <c r="I49" s="62" t="inlineStr">
+      <c r="I49" s="74" t="inlineStr">
         <is>
           <t>AI wywołuje remote beans dla smoke testów.</t>
         </is>
@@ -19759,7 +20057,7 @@
       </c>
       <c r="H50" s="28" t="n"/>
     </row>
-    <row r="51" ht="15" customHeight="1" s="51">
+    <row r="51" ht="20" customHeight="1" s="51">
       <c r="A51" s="7" t="inlineStr">
         <is>
           <t>TL.11</t>
@@ -19784,7 +20082,7 @@
       <c r="F51" s="3" t="n"/>
       <c r="G51" s="16" t="n"/>
       <c r="H51" s="28" t="n"/>
-      <c r="I51" s="62" t="inlineStr">
+      <c r="I51" s="74" t="inlineStr">
         <is>
           <t>Automatyczne zbiorcze review w pipeline.</t>
         </is>
@@ -19809,7 +20107,7 @@
       </c>
       <c r="H52" s="28" t="n"/>
     </row>
-    <row r="53" ht="15" customHeight="1" s="51">
+    <row r="53" ht="20" customHeight="1" s="51">
       <c r="A53" s="7" t="inlineStr">
         <is>
           <t>TL.15</t>
@@ -19834,7 +20132,7 @@
       <c r="F53" s="3" t="n"/>
       <c r="G53" s="16" t="n"/>
       <c r="H53" s="28" t="n"/>
-      <c r="I53" s="62" t="inlineStr">
+      <c r="I53" s="74" t="inlineStr">
         <is>
           <t>Przyrostowe wykrywanie potencjalnych bugów.</t>
         </is>
@@ -19859,7 +20157,7 @@
       </c>
       <c r="H54" s="28" t="n"/>
     </row>
-    <row r="55" ht="15" customHeight="1" s="51">
+    <row r="55" ht="20" customHeight="1" s="51">
       <c r="A55" s="7" t="inlineStr">
         <is>
           <t>TL.16</t>
@@ -19884,7 +20182,7 @@
       <c r="F55" s="3" t="n"/>
       <c r="G55" s="16" t="n"/>
       <c r="H55" s="28" t="n"/>
-      <c r="I55" s="62" t="inlineStr">
+      <c r="I55" s="74" t="inlineStr">
         <is>
           <t>Przyrostowe sprawdzenie zgodności z architekturą.</t>
         </is>
@@ -19909,7 +20207,7 @@
       </c>
       <c r="H56" s="28" t="n"/>
     </row>
-    <row r="57" ht="15" customHeight="1" s="51">
+    <row r="57" ht="20" customHeight="1" s="51">
       <c r="A57" s="7" t="inlineStr">
         <is>
           <t>TL.17</t>
@@ -19934,7 +20232,7 @@
       <c r="F57" s="3" t="n"/>
       <c r="G57" s="16" t="n"/>
       <c r="H57" s="28" t="n"/>
-      <c r="I57" s="62" t="inlineStr">
+      <c r="I57" s="74" t="inlineStr">
         <is>
           <t>Przyrostowa kontrola złożoności kodu.</t>
         </is>
@@ -19959,7 +20257,7 @@
       </c>
       <c r="H58" s="28" t="n"/>
     </row>
-    <row r="59" ht="15" customHeight="1" s="51">
+    <row r="59" ht="20" customHeight="1" s="51">
       <c r="A59" s="7" t="inlineStr">
         <is>
           <t>TL.18</t>
@@ -19984,7 +20282,7 @@
       <c r="F59" s="3" t="n"/>
       <c r="G59" s="16" t="n"/>
       <c r="H59" s="28" t="n"/>
-      <c r="I59" s="62" t="inlineStr">
+      <c r="I59" s="74" t="inlineStr">
         <is>
           <t>Sprawdzenie czy kod realizuje specyfikację.</t>
         </is>

</xml_diff>